<commit_message>
feat(F-NAR-019): ATOM-EMO.GES.001-08 Raphaël dit stop et s'éloigne
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.GES.001-08.xlsx
+++ b/stories/arbres/ATOM-EMO.GES.001-08.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Les chatouilles du canapé</t>
+          <t>Raphaël dit stop et s'éloigne</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>salon</t>
+          <t>salon, plinthe, toupie rouge, sol, fenêtre, bois, cire, trait d'or</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Mila, Aniss, papa</t>
+          <t>Raphaël, Victorino, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Mila joue sur le canapé. Aniss la chatouille trop. Mila dit stop, s'éloigne, rejoint papa. Elle goûte un morceau d'orange.</t>
+          <t>Un trait d'or file le long du bois. Sur le bois, un éclat de plinthe luit. Raphaël veut jouer, maintenant. Victorino chatouille trop. Ventre trop vite. Sourire parti. Papa s'accroupit. Raphaël dit stop, recule d'un pas. Merci vécu. Deuxième ruse : Victorino chatouille trop près du ventre. Un éclat de plinthe tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La lampe est basse et orange. Le canapé est une montagne de coussins. Dehors, une clochette de vélo passe. Le journal de papa froisse tout bas. Tu as entendu la clochette, Mila ? Oui, papa. Loin. C'est un vélo, dans la rue. Le salon sent l'orange épluchée. Une pelure brille dans l'assiette. En ce moment, Mila joue. Aniss joue avec elle. Ils sont sur le canapé. Aniss la chatouille trop. Mila est gênée. Les chatouilles durent trop. Son ventre bouge trop vite. Ses épaules montent. Je n'aime pas. C'est trop. Stop. Mila recule d'un pas. Elle peut s'éloigner. Elle s'éloigne vers le canapé. Papa est l'adulte près du canapé. Papa, c'était trop. J'ai entendu stop. Bravo, Mila. Tu as quitté le jeu. Tu es venue me le dire. Tu veux un morceau d'orange ? Oui, papa. Mila prend la main de papa. Elle souffle. Ses épaules descendent. Dire stop, c'est permis. On s'éloigne. On va vers un adulte. Aniss s'assoit plus loin. Il feuillette un livre d'images. Le salon redevient calme. Papa donne un quartier d'orange. Il est froid et sucré. C'est sucré, papa. Oui. Un peu sucré. Le jus brille sur son doigt. Mila le lèche. On reste près du canapé ? Oui, papa. La clochette est loin, maintenant. Le journal ne froisse plus. Mila pose sa tête contre papa.</t>
+          <t>Un trait d'or file le long du bois. Il est chaud, papa. Tu le vois, le trait, Raphaël ? Oui, papa. Le bois de la plinthe sent la cire. Ça sent la cire, ce soir. Oui, maman. La fenêtre laisse un air tiède. Tu sens l'air, Raphaël ? Oui, il est tiède. Une toupie rouge attend sur le sol. Elle a des ronds peints. Elle est rouge, maman. Tu la vois, la toupie ? Oui. Papa pose un doigt sur le bois. Toc, toc, contre la plinthe. Tu entends le bois, Raphaël ? Oui, il sonne. Sur le bois, un éclat de plinthe luit. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Le soleil le touche. Raphaël pose la paume près du bois. La plinthe est lisse, un peu froide. Elle est froide. Tu la touches, Raphaël ? Oui. En ce moment, Raphaël prend la toupie. Je veux jouer, maintenant ! Tout de suite ? Oui, papa. Les doigts serrent le bois peint. Tu la fais tourner ? Oui, maman. Victorino arrive près de la toupie. Il avance les doigts trop vite. Des chatouilles ! Tu viens, Victorino ? Oui. Victorino chatouille le ventre de Raphaël. Les doigts vont trop fort, trop longtemps. Oh. Je te tiens. Raphaël sent son ventre bouger trop vite. Le sourire de Raphaël disparaît. Dans son ventre, ça se bouscule. L'envie et la gêne se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Victorino, Raphaël ? Oui, papa. Tes mains sont froides, Raphaël ? Un peu, maman. L'éclat de plinthe tremble, puis tient.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La lampe est basse et orange. Le canapé est une montagne de coussins. Dehors, une clochette de vélo passe. Le journal de papa froisse tout bas. Tu as entendu la clochette, Mila ? Oui, papa. Loin. C'est un vélo, dans la rue. Le salon sent l'orange épluchée. Une pelure brille dans l'assiette. En ce moment, Mila joue. Aniss joue avec elle. Ils sont sur le canapé. Aniss la chatouille trop. Mila est gênée. Les chatouilles durent trop. Son ventre bouge trop vite. Ses épaules montent. Je n'aime pas. C'est trop. Stop. Mila recule d'un pas. Elle peut s'éloigner. Elle s'éloigne vers le canapé. Papa est l'adulte près du canapé. Papa, c'était trop. J'ai entendu stop. Bravo, Mila. Tu as quitté le jeu. Tu es venue me le dire. Tu veux un morceau d'orange ? Oui, papa. Mila prend la main de papa. Elle souffle. Ses épaules descendent. Dire stop, c'est permis. On s'éloigne. On va vers un adulte. Aniss s'assoit plus loin. Il feuillette un livre d'images. Le salon redevient calme. Papa donne un quartier d'orange. Il est froid et sucré. C'est sucré, papa. Oui. Un peu sucré. Le jus brille sur son doigt. Mila le lèche. On reste près du canapé ? Oui, papa. La clochette est loin, maintenant. Le journal ne froisse plus. Mila pose sa tête contre papa.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un trait d'or file le long du bois. Il est chaud, papa. Tu le vois, le trait, Raphaël ? Oui, papa. Le bois de la plinthe sent la cire. Ça sent la cire, ce soir. Oui, maman. La fenêtre laisse un air tiède. Tu sens l'air, Raphaël ? Oui, il est tiède. Une toupie rouge attend sur le sol. Elle a des ronds peints. Elle est rouge, maman. Tu la vois, la toupie ? Oui. Papa pose un doigt sur le bois. Toc, toc, contre la plinthe. Tu entends le bois, Raphaël ? Oui, il sonne. Sur le bois, un &lt;emphasis level="moderate"&gt;éclat de plinthe&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Le soleil le touche. Raphaël pose la paume près du bois. La plinthe est lisse, un peu froide. Elle est froide. Tu la touches, Raphaël ? Oui. En ce moment, Raphaël prend la toupie. Je veux jouer, maintenant ! Tout de suite ? Oui, papa. Les doigts serrent le bois peint. Tu la fais tourner ? Oui, maman. Victorino arrive près de la toupie. Il avance les doigts trop vite. Des chatouilles ! Tu viens, Victorino ? Oui. Victorino chatouille le ventre de Raphaël. Les doigts vont trop fort, trop longtemps. Oh. Je te tiens. Raphaël sent son ventre bouger trop vite. Le sourire de Raphaël disparaît. Dans son ventre, ça se bouscule. L'envie et la gêne se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Victorino, Raphaël ? Oui, papa. Tes mains sont froides, Raphaël ? Un peu, maman. L'éclat de plinthe tremble, puis tient.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Hippolyte joue dans le salon. Un camarade le chatouille trop. Hippolyte sent son ventre. C'est trop. Il dit : &lt;emphasis&gt;stop&lt;/emphasis&gt;. Il recule d'un pas. Il peut s'éloigner. Il s'éloigne vers le canapé. Papa est l'adulte. Hippolyte va vers papa. Il dit : c'était trop. Papa l'écoute. Hippolyte prend la main de papa. Il souffle. Ses épaules descendent. Dire stop, c'est permis. On s'éloigne. On va vers un adulte.&lt;/slow&gt; [pause]</t>
+          <t>Un trait d'or file le long du bois. Il est chaud, papa. Tu le vois, le trait, Raphaël ? Oui, papa. Le bois de la plinthe sent la cire. Ça sent la cire, ce soir. Oui, maman. La fenêtre laisse un air tiède. Tu sens l'air, Raphaël ? Oui, il est tiède. Une toupie rouge attend sur le sol. Elle a des ronds peints. Elle est rouge, maman. Tu la vois, la toupie ? Oui. Papa pose un doigt sur le bois. Toc, toc, contre la plinthe. Tu entends le bois, Raphaël ? Oui, il sonne. Sur le bois, un &lt;emphasis&gt;éclat de plinthe&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Le soleil le touche. Raphaël pose la paume près du bois. La plinthe est lisse, un peu froide. Elle est froide. Tu la touches, Raphaël ? Oui. En ce moment, Raphaël prend la toupie. Je veux jouer, maintenant ! Tout de suite ? Oui, papa. Les doigts serrent le bois peint. Tu la fais tourner ? Oui, maman. Victorino arrive près de la toupie. Il avance les doigts trop vite. Des chatouilles ! Tu viens, Victorino ? Oui. Victorino chatouille le ventre de Raphaël. Les doigts vont trop fort, trop longtemps. Oh. Je te tiens. Raphaël sent son ventre bouger trop vite. Le sourire de Raphaël disparaît. Dans son ventre, ça se bouscule. L'envie et la gêne se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Victorino, Raphaël ? Oui, papa. Tes mains sont froides, Raphaël ? Un peu, maman. L'éclat de plinthe tremble, puis tient. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,18 +1246,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.22</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>stop</t>
+          <t>éclat de plinthe</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>560</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>300</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1324,62 +1324,71 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_jouer_maintenant; tempo=posé puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La lampe est basse et orange.
-narrateur|Le canapé est une montagne de coussins.
-narrateur|Dehors, une clochette de vélo passe.
-narrateur|Le journal de papa froisse tout bas.
-papa|Tu as entendu la clochette, Mila ?
-enfant-f|Oui, papa. Loin.
-papa|C'est un vélo, dans la rue.
-narrateur|Le salon sent l'orange épluchée.
-narrateur|Une pelure brille dans l'assiette.
-narrateur|En ce moment, Mila joue.
-narrateur|Aniss joue avec elle.
-narrateur|Ils sont sur le canapé.
-narrateur|Aniss la chatouille trop.
-narrateur|Mila est gênée.
-narrateur|Les chatouilles durent trop.
-narrateur|Son ventre bouge trop vite.
-narrateur|Ses épaules montent.
-enfant-f|Je n'aime pas.
-enfant-f|C'est trop.
-enfant-f|Stop.
-narrateur|Mila recule d'un pas.
-narrateur|Elle peut s'éloigner.
-narrateur|Elle s'éloigne vers le canapé.
-narrateur|Papa est l'adulte près du canapé.
-enfant-f|Papa, c'était trop.
-papa|J'ai entendu stop.
-papa|Bravo, Mila.
-papa|Tu as quitté le jeu.
-papa|Tu es venue me le dire.
-papa|Tu veux un morceau d'orange ?
-enfant-f|Oui, papa.
-narrateur|Mila prend la main de papa.
-narrateur|Elle souffle.
-narrateur|Ses épaules descendent.
-papa|Dire stop, c'est permis.
-papa|On s'éloigne.
-papa|On va vers un adulte.
-narrateur|Aniss s'assoit plus loin.
-narrateur|Il feuillette un livre d'images.
-narrateur|Le salon redevient calme.
-narrateur|Papa donne un quartier d'orange.
-narrateur|Il est froid et sucré.
-enfant-f|C'est sucré, papa.
-papa|Oui. Un peu sucré.
-narrateur|Le jus brille sur son doigt.
-narrateur|Mila le lèche.
-papa|On reste près du canapé ?
-enfant-f|Oui, papa.
-narrateur|La clochette est loin, maintenant.
-narrateur|Le journal ne froisse plus.
-narrateur|Mila pose sa tête contre papa.</t>
+          <t>narrateur|Un trait d'or file le long du bois.
+enfant-m|Il est chaud, papa.
+papa|Tu le vois, le trait, Raphaël ?
+enfant-m|Oui, papa.
+narrateur|Le bois de la plinthe sent la cire.
+maman|Ça sent la cire, ce soir.
+enfant-m|Oui, maman.
+narrateur|La fenêtre laisse un air tiède.
+papa|Tu sens l'air, Raphaël ?
+enfant-m|Oui, il est tiède.
+narrateur|Une toupie rouge attend sur le sol.
+narrateur|Elle a des ronds peints.
+enfant-m|Elle est rouge, maman.
+maman|Tu la vois, la toupie ?
+enfant-m|Oui.
+narrateur|Papa pose un doigt sur le bois.
+narrateur|Toc, toc, contre la plinthe.
+papa|Tu entends le bois, Raphaël ?
+enfant-m|Oui, il sonne.
+narrateur|Sur le bois, un éclat de plinthe luit.
+enfant-m|Il brille, maman.
+maman|Tu le vois, le petit point ?
+enfant-m|Oui, un petit point.
+papa|Le soleil le touche.
+narrateur|Raphaël pose la paume près du bois.
+narrateur|La plinthe est lisse, un peu froide.
+enfant-m|Elle est froide.
+maman|Tu la touches, Raphaël ?
+enfant-m|Oui.
+narrateur|En ce moment, Raphaël prend la toupie.
+enfant-m|Je veux jouer, maintenant !
+papa|Tout de suite ?
+enfant-m|Oui, papa.
+narrateur|Les doigts serrent le bois peint.
+maman|Tu la fais tourner ?
+enfant-m|Oui, maman.
+narrateur|Victorino arrive près de la toupie.
+narrateur|Il avance les doigts trop vite.
+copain|Des chatouilles !
+enfant-m|Tu viens, Victorino ?
+copain|Oui.
+narrateur|Victorino chatouille le ventre de Raphaël.
+narrateur|Les doigts vont trop fort, trop longtemps.
+enfant-m|Oh.
+copain|Je te tiens.
+narrateur|Raphaël sent son ventre bouger trop vite.
+narrateur|Le sourire de Raphaël disparaît.
+narrateur|Dans son ventre, ça se bouscule.
+narrateur|L'envie et la gêne se heurtent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois Victorino, Raphaël ?
+enfant-m|Oui, papa.
+maman|Tes mains sont froides, Raphaël ?
+enfant-m|Un peu, maman.
+narrateur|L'éclat de plinthe tremble, puis tient.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1411,17 +1420,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>C'est trop pour Mila. Que dit-elle ?</t>
+          <t>C'est trop pour Raphaël. Que dit-il ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>C'est trop pour Mila. Que dit-elle ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;C'est trop pour &lt;emphasis level="moderate"&gt;Raphaël&lt;/emphasis&gt;. Que dit-il ?&lt;/prosody&gt;&lt;break time="780ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;C'est trop pour Hippolyte. Que dit-il ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;C'est trop pour &lt;emphasis&gt;Raphaël&lt;/emphasis&gt;. Que dit-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1446,7 +1455,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Hippolyte dit stop. Puis il va où ?</t>
+          <t>Raphaël dit stop. Puis il va où ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1484,7 +1493,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1495,7 +1504,7 @@
         <v>0.8</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.36</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1510,34 +1519,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Raphaël</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>780</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>360</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.3</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1552,7 +1565,7 @@
         <v>0.8</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1562,12 +1575,13 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=c_est_trop_pour_raphael_que_dit_il; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|C'est trop pour Mila. Que dit-elle ?</t>
+          <t>narrateur|C'est trop pour Raphaël.
+narrateur|Que dit-il ?</t>
         </is>
       </c>
     </row>
@@ -1594,17 +1608,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Mila a dit stop. Elle a pu s'éloigner. Elle a rejoint papa, l'adulte. Tu as dit stop. Bravo. Tu restes près de moi ? Oui. L'orange est sucrée. La lampe est encore orange.</t>
+          <t>Raphaël veut la toupie, tout de suite. Je tourne, maintenant ! Victorino chatouille trop, trop près. Les mots se bousculent dans sa bouche. Viens. Victorino avance d'un pas. Stop. Raphaël recule d'un pas. Le sourire ne revient pas. Raphaël refuse de rester collé. Il referme la bouche. Personne ne parle. Il observe la toupie, un instant. Il écoute le bois de la plinthe. Tu veux la toupie avec Victorino ? Papa reste à la même hauteur. Tu restes un peu loin ? Victorino ne dit rien, d'abord. Il ouvre les mains, puis les baisse. Je m'arrête. D'accord. Merci, Raphaël. Papa a vu les deux, près du bois. La cire colle un peu, sous les doigts. Elle est tiède. Raphaël essuie la toupie du plat de la main. Victorino reste un pas plus loin. La toupie part sans coller, cette fois. Elle tourne ! Oui. Tu la vois, la toupie ? Oui, papa. Tu pousses, Victorino ? J'y vais. Raphaël lance, sans se presser. Victorino suit la toupie des yeux. La toupie danse une fois. Un. Deux. Le ventre de Raphaël se desserre. Les épaules se relèvent un peu. On reste près de la plinthe ? Oui. Tes mains sont au chaud ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Mila a dit stop. Elle a pu s'éloigner. Elle a rejoint papa, l'adulte. Tu as dit stop. Bravo. Tu restes près de moi ? Oui. L'orange est sucrée. La lampe est encore orange.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël veut la toupie, tout de suite. Je tourne, maintenant ! Victorino chatouille trop, trop près. Les mots se bousculent dans sa bouche. Viens. Victorino avance d'un pas. Stop. Raphaël recule d'un pas. Le sourire ne revient pas. Raphaël refuse de rester collé. Il referme la bouche. Personne ne parle. Il observe la toupie, un instant. Il écoute le bois de la plinthe. Tu veux la toupie avec Victorino ? Papa reste à la même hauteur. Tu restes un peu loin ? Victorino ne dit rien, d'abord. Il ouvre les mains, puis les baisse. Je m'arrête. D'accord. Merci, Raphaël. Papa a vu les deux, près du bois. La cire colle un peu, sous les doigts. Elle est tiède. Raphaël essuie la toupie du plat de la main. Victorino reste un pas plus loin. La toupie part sans coller, cette fois. Elle tourne ! Oui. Tu la vois, la toupie ? Oui, papa. Tu pousses, Victorino ? J'y vais. Raphaël lance, sans se presser. Victorino suit la toupie des yeux. La toupie danse une fois. Un. Deux. Le ventre de Raphaël se desserre. Les épaules se relèvent un peu. On reste près de la plinthe ? Oui. Tes mains sont au chaud ? Un peu, maman.&lt;/prosody&gt;&lt;break time="620ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Hippolyte a dit &lt;emphasis&gt;stop&lt;/emphasis&gt;. Il a pu s'éloigner. Il rejoint papa, l'adulte.&lt;/slow&gt; [pause]</t>
+          <t>Raphaël veut la toupie, tout de suite. Je tourne, maintenant ! Victorino chatouille trop, trop près. Les mots se bousculent dans sa bouche. Viens. Victorino avance d'un pas. Stop. Raphaël recule d'un pas. Le sourire ne revient pas. Raphaël refuse de rester collé. Il referme la bouche. Personne ne parle. Il observe la toupie, un instant. Il écoute le bois de la plinthe. Tu veux la toupie avec Victorino ? Papa reste à la même hauteur. Tu restes un peu loin ? Victorino ne dit rien, d'abord. Il ouvre les mains, puis les baisse. Je m'arrête. D'accord. Merci, Raphaël. Papa a vu les deux, près du bois. La cire colle un peu, sous les doigts. Elle est tiède. Raphaël essuie la toupie du plat de la main. Victorino reste un pas plus loin. La toupie part sans coller, cette fois. Elle tourne ! Oui. Tu la vois, la toupie ? Oui, papa. Tu pousses, Victorino ? J'y vais. Raphaël lance, sans se presser. Victorino suit la toupie des yeux. La toupie danse une fois. Un. Deux. Le ventre de Raphaël se desserre. Les épaules se relèvent un peu. On reste près de la plinthe ? Oui. Tes mains sont au chaud ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1651,18 +1665,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.24</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1692,23 +1706,23 @@
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>620</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>310</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.33</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1717,10 +1731,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1729,24 +1743,60 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_dit_stop_il_recule; tempo=posé; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Mila a dit stop.
-narrateur|Elle a pu s'éloigner.
-narrateur|Elle a rejoint papa, l'adulte.
-papa|Tu as dit stop.
-papa|Bravo.
-papa|Tu restes près de moi ?
-enfant-f|Oui.
-narrateur|L'orange est sucrée.
-narrateur|La lampe est encore orange.</t>
+          <t>narrateur|Raphaël veut la toupie, tout de suite.
+enfant-m|Je tourne, maintenant !
+narrateur|Victorino chatouille trop, trop près.
+narrateur|Les mots se bousculent dans sa bouche.
+copain|Viens.
+narrateur|Victorino avance d'un pas.
+enfant-m|Stop.
+narrateur|Raphaël recule d'un pas.
+narrateur|Le sourire ne revient pas.
+narrateur|Raphaël refuse de rester collé.
+narrateur|Il referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Il observe la toupie, un instant.
+narrateur|Il écoute le bois de la plinthe.
+papa|Tu veux la toupie avec Victorino ?
+narrateur|Papa reste à la même hauteur.
+enfant-m|Tu restes un peu loin ?
+narrateur|Victorino ne dit rien, d'abord.
+narrateur|Il ouvre les mains, puis les baisse.
+copain|Je m'arrête.
+enfant-m|D'accord.
+papa|Merci, Raphaël.
+narrateur|Papa a vu les deux, près du bois.
+maman|La cire colle un peu, sous les doigts.
+enfant-m|Elle est tiède.
+narrateur|Raphaël essuie la toupie du plat de la main.
+narrateur|Victorino reste un pas plus loin.
+narrateur|La toupie part sans coller, cette fois.
+enfant-m|Elle tourne !
+copain|Oui.
+papa|Tu la vois, la toupie ?
+enfant-m|Oui, papa.
+maman|Tu pousses, Victorino ?
+copain|J'y vais.
+narrateur|Raphaël lance, sans se presser.
+narrateur|Victorino suit la toupie des yeux.
+narrateur|La toupie danse une fois.
+copain|Un.
+enfant-m|Deux.
+narrateur|Le ventre de Raphaël se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|On reste près de la plinthe ?
+enfant-m|Oui.
+maman|Tes mains sont au chaud ?
+enfant-m|Un peu, maman.</t>
         </is>
       </c>
     </row>
@@ -1773,17 +1823,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Mila reste près du canapé. Papa lui parle tout bas. Ton ventre allait trop vite. Tu as écouté. Tu es plus calme, maintenant ? Oui, papa. La pelure brille encore. Mila souffle une dernière fois. Le livre d'Aniss fait un petit bruit. Une page se tourne. Toi, tu restes ici. Près de moi.</t>
+          <t>Maman approche la toupie. Elle la tend vers Victorino. Je joue, maintenant ! Victorino court trop, tout de suite. Il chatouille trop près du ventre. Avec moi ! La toupie penche vers Victorino. Elle penche ! Raphaël avance les mains, trop vite. Puis il s'arrête net. Raphaël refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe la toupie, un instant. Il écoute le bois de la plinthe. Sur le bois, un éclat de plinthe luit. Là, sur le bois. Stop. Raphaël recule d'un pas. Victorino ne dit rien. Il souffle, puis recule aussi. Oui. On tient la toupie ? Oui, papa. La toupie sent le bois peint. Le bois est là, un peu tiède. Raphaël la pousse vers Victorino. Victorino la rend, sans se coller. Vzz. Vzz. La toupie est bien calme ? Oui, papa. La cire est chaude, Victorino ? Un peu. Ils poussent la toupie, à un pas. Le sol chatouille les genoux. C'est plus facile. La plinthe est calme ? Oui, papa. Un trait d'or passe sur le bois. Il allume la plinthe.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Mila reste près du canapé. Papa lui parle tout bas. Ton ventre allait trop vite. Tu as écouté. Tu es plus calme, maintenant ? Oui, papa. La pelure brille encore. Mila souffle une dernière fois. Le livre d'Aniss fait un petit bruit. Une page se tourne. Toi, tu restes ici. Près de moi.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman approche la toupie. Elle la tend vers Victorino. Je joue, maintenant ! Victorino court trop, tout de suite. Il chatouille trop près du ventre. Avec moi ! La toupie penche vers Victorino. Elle penche ! Raphaël avance les mains, trop vite. Puis il s'arrête net. Raphaël refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe la toupie, un instant. Il écoute le bois de la plinthe. Sur le bois, un &lt;emphasis level="moderate"&gt;éclat de plinthe&lt;/emphasis&gt; luit. Là, sur le bois. Stop. Raphaël recule d'un pas. Victorino ne dit rien. Il souffle, puis recule aussi. Oui. On tient la toupie ? Oui, papa. La toupie sent le bois peint. Le bois est là, un peu tiède. Raphaël la pousse vers Victorino. Victorino la rend, sans se coller. Vzz. Vzz. La toupie est bien calme ? Oui, papa. La cire est chaude, Victorino ? Un peu. Ils poussent la toupie, à un pas. Le sol chatouille les genoux. C'est plus facile. La plinthe est calme ? Oui, papa. Un trait d'or passe sur le bois. Il allume la plinthe.&lt;/prosody&gt;&lt;break time="480ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Hippolyte reste près du canapé. Papa lui parle tout bas.&lt;/slow&gt; [pause]</t>
+          <t>Maman approche la toupie. Elle la tend vers Victorino. Je joue, maintenant ! Victorino court trop, tout de suite. Il chatouille trop près du ventre. Avec moi ! La toupie penche vers Victorino. Elle penche ! Raphaël avance les mains, trop vite. Puis il s'arrête net. Raphaël refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe la toupie, un instant. Il écoute le bois de la plinthe. Sur le bois, un &lt;emphasis&gt;éclat de plinthe&lt;/emphasis&gt; luit. Là, sur le bois. Stop. Raphaël recule d'un pas. Victorino ne dit rien. Il souffle, puis recule aussi. Oui. On tient la toupie ? Oui, papa. La toupie sent le bois peint. Le bois est là, un peu tiède. Raphaël la pousse vers Victorino. Victorino la rend, sans se coller. Vzz. Vzz. La toupie est bien calme ? Oui, papa. La cire est chaude, Victorino ? Un peu. Ils poussent la toupie, à un pas. Le sol chatouille les genoux. C'est plus facile. La plinthe est calme ? Oui, papa. Un trait d'or passe sur le bois. Il allume la plinthe. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1830,18 +1880,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1862,28 +1912,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de plinthe</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>480</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>280</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1892,10 +1946,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1904,23 +1958,56 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=victorino_chatouille_trop_pres_il_s_arrete; tempo=un peu vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Mila reste près du canapé.
-narrateur|Papa lui parle tout bas.
-papa|Ton ventre allait trop vite.
-papa|Tu as écouté.
-papa|Tu es plus calme, maintenant ?
-enfant-f|Oui, papa.
-narrateur|La pelure brille encore.
-narrateur|Mila souffle une dernière fois.
-narrateur|Le livre d'Aniss fait un petit bruit.
-narrateur|Une page se tourne.
-papa|Toi, tu restes ici.
-papa|Près de moi.</t>
+          <t>narrateur|Maman approche la toupie.
+narrateur|Elle la tend vers Victorino.
+enfant-m|Je joue, maintenant !
+narrateur|Victorino court trop, tout de suite.
+narrateur|Il chatouille trop près du ventre.
+copain|Avec moi !
+narrateur|La toupie penche vers Victorino.
+enfant-m|Elle penche !
+narrateur|Raphaël avance les mains, trop vite.
+narrateur|Puis il s'arrête net.
+narrateur|Raphaël refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Il observe la toupie, un instant.
+narrateur|Il écoute le bois de la plinthe.
+narrateur|Sur le bois, un éclat de plinthe luit.
+enfant-m|Là, sur le bois.
+enfant-m|Stop.
+narrateur|Raphaël recule d'un pas.
+narrateur|Victorino ne dit rien.
+narrateur|Il souffle, puis recule aussi.
+copain|Oui.
+papa|On tient la toupie ?
+enfant-m|Oui, papa.
+narrateur|La toupie sent le bois peint.
+narrateur|Le bois est là, un peu tiède.
+narrateur|Raphaël la pousse vers Victorino.
+narrateur|Victorino la rend, sans se coller.
+enfant-m|Vzz.
+copain|Vzz.
+papa|La toupie est bien calme ?
+enfant-m|Oui, papa.
+maman|La cire est chaude, Victorino ?
+copain|Un peu.
+narrateur|Ils poussent la toupie, à un pas.
+narrateur|Le sol chatouille les genoux.
+enfant-m|C'est plus facile.
+papa|La plinthe est calme ?
+enfant-m|Oui, papa.
+maman|Un trait d'or passe sur le bois.
+enfant-m|Il allume la plinthe.</t>
         </is>
       </c>
     </row>
@@ -1947,17 +2034,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit stop. Je me suis éloignée. Je suis allée vers papa. Bravo.</t>
+          <t>Ils restent près de la plinthe. Maman essuie un peu de cire. La toupie a penché, papa. Tu l'as vue, toi ? Oui, près de la plinthe. On est bien, ici. Raphaël tapote le bois du doigt. Il a une trace de cire. Tu la vois, la trace ? Oui, maman. La toupie est restée, Raphaël. Oui, avec Victorino. La toupie est restée. Ça sent la cire, un peu tiède. Et le bois, maman. Oui, dans l'air. La toupie reste près du sol. Un éclat de plinthe tient sur le bois.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit stop. Je me suis éloignée. Je suis allée vers papa. Bravo.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la plinthe. Maman essuie un peu de cire. La toupie a penché, papa. Tu l'as vue, toi ? Oui, près de la plinthe. On est bien, ici. Raphaël tapote le bois du doigt. Il a une trace de cire. Tu la vois, la trace ? Oui, maman. La toupie est restée, Raphaël. Oui, avec Victorino. La toupie est restée. Ça sent la cire, un peu tiède. Et le bois, maman. Oui, dans l'air. La toupie reste près du sol. Un &lt;emphasis level="moderate"&gt;éclat de plinthe&lt;/emphasis&gt; tient sur le bois.&lt;/prosody&gt;&lt;break time="980ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la plinthe. Maman essuie un peu de cire. La toupie a penché, papa. Tu l'as vue, toi ? Oui, près de la plinthe. On est bien, ici. Raphaël tapote le bois du doigt. Il a une trace de cire. Tu la vois, la trace ? Oui, maman. La toupie est restée, Raphaël. Oui, avec Victorino. La toupie est restée. Ça sent la cire, un peu tiède. Et le bois, maman. Oui, dans l'air. La toupie reste près du sol. Un &lt;emphasis&gt;éclat de plinthe&lt;/emphasis&gt; tient sur le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2004,7 +2091,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2012,7 +2099,7 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.36</v>
@@ -2024,12 +2111,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2038,14 +2125,18 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de plinthe</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>980</v>
       </c>
       <c r="AK6" s="2" t="n">
         <v>380</v>
@@ -2057,11 +2148,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.29</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2070,27 +2161,45 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bois; tempo=très posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|J'ai dit stop.
-enfant-f|Je me suis éloignée.
-enfant-f|Je suis allée vers papa.
-papa|Bravo.</t>
+          <t>narrateur|Ils restent près de la plinthe.
+narrateur|Maman essuie un peu de cire.
+enfant-m|La toupie a penché, papa.
+papa|Tu l'as vue, toi ?
+enfant-m|Oui, près de la plinthe.
+maman|On est bien, ici.
+narrateur|Raphaël tapote le bois du doigt.
+enfant-m|Il a une trace de cire.
+maman|Tu la vois, la trace ?
+enfant-m|Oui, maman.
+papa|La toupie est restée, Raphaël.
+enfant-m|Oui, avec Victorino.
+copain|La toupie est restée.
+narrateur|Ça sent la cire, un peu tiède.
+enfant-m|Et le bois, maman.
+maman|Oui, dans l'air.
+narrateur|La toupie reste près du sol.
+narrateur|Un éclat de plinthe tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -2111,7 +2220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2168,6 +2277,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>